<commit_message>
fix(design-zones): band 시각비교에서 dtype 제외 + 풀 P&L 예시본
결함 7: zone_findings 가 band-spec(대표셀 1개)의 dtype 으로 비교 → 한 band 에 값(Q1~Q4)과
수식(누계 SUM)이 정당하게 혼재할 때 수식셀을 drift 오탐(예: G13 dtype f vs spec n). band
시각 비교에서 dtype 제외(formula↔value 혼재 허용), quotePrefix/numFmt/font/fill/align 은 유지.
formula 석화 검출은 golden 경로 담당(band-spec 아님).

예시본 강화: 풀 P&L 10라인(매출~당기순이익) + 소계 3행(SUM·상단보더) + 실적 Q1~Q4·누계
+ 전망FY + 달성%(IF 가드). 9블록(hdr/data/total × actual/fcst/ratio). 라우터 clean PASS,
verify_xlsx 에러셀 0.

게이트: selftest ALL PASS / unittest 83 OK.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/example_design_zones_mixed.xlsx
+++ b/example_design_zones_mixed.xlsx
@@ -16,10 +16,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0;(#,##0)"/>
+    <numFmt numFmtId="165" formatCode="0.0%;(0.0%)"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,12 +35,23 @@
     </font>
     <font>
       <name val="맑은 고딕"/>
+      <color rgb="005B616B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
       <b val="1"/>
       <color rgb="00111418"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="맑은 고딕"/>
+      <color rgb="00111418"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
       <color rgb="00111418"/>
       <sz val="10"/>
     </font>
@@ -57,7 +69,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -70,22 +82,42 @@
         <color rgb="0012404A"/>
       </bottom>
     </border>
+    <border>
+      <top style="thin">
+        <color rgb="00D8DCE0"/>
+      </top>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -453,25 +485,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col hidden="1" width="13" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>FY2026 손익 — 실적/전망 (design-zones 예시)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+          <t>FY2026 손익계산서 — 실적·전망 (design-zones 예시)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>단위: 백만원 / 실적 Q1~Q4·누계, 전망 FY, 달성률</t>
+        </is>
+      </c>
+    </row>
     <row r="3"/>
     <row r="4" hidden="1">
       <c r="A4" t="inlineStr">
@@ -489,9 +530,14 @@
           <t>actual</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>fcst</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>ratio</t>
         </is>
       </c>
     </row>
@@ -501,29 +547,44 @@
           <t>hdr</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>실적 Q1</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>실적 Q2</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>전망 Q3</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>전망 Q4</t>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>누계</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>전망FY</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>달성%</t>
         </is>
       </c>
     </row>
@@ -533,85 +594,349 @@
           <t>data</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>매출</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>1200</v>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>1350</v>
-      </c>
-      <c r="E6" s="4" t="n">
-        <v>1500</v>
-      </c>
-      <c r="F6" s="4" t="n">
-        <v>1620</v>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>매출액</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>3200</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>3450</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>3600</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>3850</v>
+      </c>
+      <c r="G6" s="5">
+        <f>SUM(C6:F6)</f>
+        <v/>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>14500</v>
+      </c>
+      <c r="I6" s="6">
+        <f>IF(H6=0,"NA",G6/H6)</f>
+        <v/>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>매출원가</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n">
-        <v>-700</v>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>-790</v>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>-880</v>
-      </c>
-      <c r="F7" s="4" t="n">
-        <v>-950</v>
+      <c r="C7" s="5" t="n">
+        <v>-1900</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>-2050</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>-2150</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>-2300</v>
+      </c>
+      <c r="G7" s="5">
+        <f>SUM(C7:F7)</f>
+        <v/>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>-8600</v>
+      </c>
+      <c r="I7" s="6">
+        <f>IF(H7=0,"NA",G7/H7)</f>
+        <v/>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="3" t="inlineStr">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>매출총이익</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n">
-        <v>500</v>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>560</v>
-      </c>
-      <c r="E8" s="4" t="n">
-        <v>620</v>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>670</v>
+      <c r="C8" s="8">
+        <f>C6+C7</f>
+        <v/>
+      </c>
+      <c r="D8" s="8">
+        <f>D6+D7</f>
+        <v/>
+      </c>
+      <c r="E8" s="8">
+        <f>E6+E7</f>
+        <v/>
+      </c>
+      <c r="F8" s="8">
+        <f>F6+F7</f>
+        <v/>
+      </c>
+      <c r="G8" s="8">
+        <f>SUM(C8:F8)</f>
+        <v/>
+      </c>
+      <c r="H8" s="8">
+        <f>H6+H7</f>
+        <v/>
+      </c>
+      <c r="I8" s="9">
+        <f>IF(H8=0,"NA",G8/H8)</f>
+        <v/>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="3" t="inlineStr">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>판매비</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>-420</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>-440</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>-460</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>-480</v>
+      </c>
+      <c r="G9" s="5">
+        <f>SUM(C9:F9)</f>
+        <v/>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>-1850</v>
+      </c>
+      <c r="I9" s="6">
+        <f>IF(H9=0,"NA",G9/H9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>관리비</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>-300</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>-310</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>-320</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>-330</v>
+      </c>
+      <c r="G10" s="5">
+        <f>SUM(C10:F10)</f>
+        <v/>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>-1300</v>
+      </c>
+      <c r="I10" s="6">
+        <f>IF(H10=0,"NA",G10/H10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>연구개발비</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>-180</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>-190</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>-200</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>-210</v>
+      </c>
+      <c r="G11" s="5">
+        <f>SUM(C11:F11)</f>
+        <v/>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>-820</v>
+      </c>
+      <c r="I11" s="6">
+        <f>IF(H11=0,"NA",G11/H11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>영업이익</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n">
-        <v>180</v>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>210</v>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>250</v>
-      </c>
-      <c r="F9" s="4" t="n">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>※ Q3~Q4는 전망치(잠정).</t>
+      <c r="C12" s="8">
+        <f>C8+C9+C10+C11</f>
+        <v/>
+      </c>
+      <c r="D12" s="8">
+        <f>D8+D9+D10+D11</f>
+        <v/>
+      </c>
+      <c r="E12" s="8">
+        <f>E8+E9+E10+E11</f>
+        <v/>
+      </c>
+      <c r="F12" s="8">
+        <f>F8+F9+F10+F11</f>
+        <v/>
+      </c>
+      <c r="G12" s="8">
+        <f>SUM(C12:F12)</f>
+        <v/>
+      </c>
+      <c r="H12" s="8">
+        <f>H8+H9+H10+H11</f>
+        <v/>
+      </c>
+      <c r="I12" s="9">
+        <f>IF(H12=0,"NA",G12/H12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>금융손익</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>-30</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>-28</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>-32</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>-35</v>
+      </c>
+      <c r="G13" s="5">
+        <f>SUM(C13:F13)</f>
+        <v/>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>-130</v>
+      </c>
+      <c r="I13" s="6">
+        <f>IF(H13=0,"NA",G13/H13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>법인세비용</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>-60</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>-70</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>-72</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>-80</v>
+      </c>
+      <c r="G14" s="5">
+        <f>SUM(C14:F14)</f>
+        <v/>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>-300</v>
+      </c>
+      <c r="I14" s="6">
+        <f>IF(H14=0,"NA",G14/H14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>당기순이익</t>
+        </is>
+      </c>
+      <c r="C15" s="8">
+        <f>C12+C13+C14</f>
+        <v/>
+      </c>
+      <c r="D15" s="8">
+        <f>D12+D13+D14</f>
+        <v/>
+      </c>
+      <c r="E15" s="8">
+        <f>E12+E13+E14</f>
+        <v/>
+      </c>
+      <c r="F15" s="8">
+        <f>F12+F13+F14</f>
+        <v/>
+      </c>
+      <c r="G15" s="8">
+        <f>SUM(C15:F15)</f>
+        <v/>
+      </c>
+      <c r="H15" s="8">
+        <f>H12+H13+H14</f>
+        <v/>
+      </c>
+      <c r="I15" s="9">
+        <f>IF(H15=0,"NA",G15/H15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>주) 전망FY는 잠정. 달성%=누계/전망FY.</t>
         </is>
       </c>
     </row>

</xml_diff>